<commit_message>
It is now fully and correctly configured
</commit_message>
<xml_diff>
--- a/output/model_coefficients.xlsx
+++ b/output/model_coefficients.xlsx
@@ -485,13 +485,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.3096428421874478</v>
+        <v>0.3088038512849631</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02871493781288128</v>
+        <v>0.02861802877767414</v>
       </c>
       <c r="G2" t="n">
-        <v>10.78333667982946</v>
+        <v>10.79053535354191</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -517,16 +517,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-0.03357280709910466</v>
+        <v>-0.03338827135018992</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02643089190467625</v>
+        <v>0.02644027427681928</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.270210903926955</v>
+        <v>-1.26278082441071</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2040095146122849</v>
+        <v>0.2066679578712263</v>
       </c>
     </row>
     <row r="4">
@@ -549,16 +549,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>-0.1958267700932454</v>
+        <v>-0.1948833040031538</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02486415908861745</v>
+        <v>0.02478917529131924</v>
       </c>
       <c r="G4" t="n">
-        <v>-7.875865392729771</v>
+        <v>-7.86162918713706</v>
       </c>
       <c r="H4" t="n">
-        <v>3.33066907387547e-15</v>
+        <v>3.774758283725532e-15</v>
       </c>
     </row>
     <row r="5">
@@ -581,16 +581,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.2108718207264798</v>
+        <v>0.2108980808682997</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02748863692396171</v>
+        <v>0.02750670885528215</v>
       </c>
       <c r="G5" t="n">
-        <v>7.671235983876403</v>
+        <v>7.667150656598219</v>
       </c>
       <c r="H5" t="n">
-        <v>1.709743457922741e-14</v>
+        <v>1.754152378907747e-14</v>
       </c>
     </row>
     <row r="6">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.1048096038056194</v>
+        <v>0.1045204919093416</v>
       </c>
       <c r="F6" t="n">
-        <v>0.02042459866803516</v>
+        <v>0.02018079419821422</v>
       </c>
       <c r="G6" t="n">
-        <v>5.131537980450829</v>
+        <v>5.179206074724816</v>
       </c>
       <c r="H6" t="n">
-        <v>2.873842190886933e-07</v>
+        <v>2.2283220579844e-07</v>
       </c>
     </row>
     <row r="7">
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>-0.2233471510629757</v>
+        <v>-0.2177505108852633</v>
       </c>
       <c r="F7" t="n">
-        <v>0.02295438650997957</v>
+        <v>0.02270833977707443</v>
       </c>
       <c r="G7" t="n">
-        <v>-9.73004227127325</v>
+        <v>-9.589010601977511</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -677,16 +677,16 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.1468258324720093</v>
+        <v>0.09868569573122142</v>
       </c>
       <c r="F8" t="n">
-        <v>0.02981671891931801</v>
+        <v>0.02539458851374513</v>
       </c>
       <c r="G8" t="n">
-        <v>4.924278652670861</v>
+        <v>3.886091545603132</v>
       </c>
       <c r="H8" t="n">
-        <v>8.467210970142247e-07</v>
+        <v>0.0001018711034188602</v>
       </c>
     </row>
     <row r="9">
@@ -709,16 +709,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-0.02486767235423624</v>
+        <v>-0.02949116436650812</v>
       </c>
       <c r="F9" t="n">
-        <v>0.02814473713806025</v>
+        <v>0.02326896014092567</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.8835638517911051</v>
+        <v>-1.26740362210563</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3769316997897563</v>
+        <v>0.2050110053263867</v>
       </c>
     </row>
     <row r="10">
@@ -779,13 +779,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1.141915097905106</v>
+        <v>1.139818198694039</v>
       </c>
       <c r="F11" t="n">
-        <v>0.04690454711497385</v>
+        <v>0.04683711912338642</v>
       </c>
       <c r="G11" t="n">
-        <v>24.34550951065923</v>
+        <v>24.33578793919834</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -811,13 +811,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1.111077498796915</v>
+        <v>1.109278981558698</v>
       </c>
       <c r="F12" t="n">
-        <v>0.05058504392579328</v>
+        <v>0.05050849613980428</v>
       </c>
       <c r="G12" t="n">
-        <v>21.96454549698261</v>
+        <v>21.96222549304027</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1.080269919657951</v>
+        <v>1.079201533537488</v>
       </c>
       <c r="F13" t="n">
-        <v>0.05307644808405824</v>
+        <v>0.05300199089745022</v>
       </c>
       <c r="G13" t="n">
-        <v>20.3530936721077</v>
+        <v>20.36152822268879</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -875,13 +875,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1.1759636714772</v>
+        <v>1.174850803484254</v>
       </c>
       <c r="F14" t="n">
-        <v>0.04921505939495964</v>
+        <v>0.04915064663729472</v>
       </c>
       <c r="G14" t="n">
-        <v>23.8943869195806</v>
+        <v>23.90305893898237</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -907,13 +907,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1.235073843452108</v>
+        <v>1.234141416068745</v>
       </c>
       <c r="F15" t="n">
-        <v>0.04808664518534514</v>
+        <v>0.04802530269259177</v>
       </c>
       <c r="G15" t="n">
-        <v>25.68434205933801</v>
+        <v>25.69773321248471</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -977,13 +977,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1.309761032925761</v>
+        <v>1.307927280807434</v>
       </c>
       <c r="F17" t="n">
-        <v>0.08065045173657748</v>
+        <v>0.08069810704829898</v>
       </c>
       <c r="G17" t="n">
-        <v>16.23997144104654</v>
+        <v>16.2076575105834</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1009,13 +1009,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.9938274628425283</v>
+        <v>0.9922991576720597</v>
       </c>
       <c r="F18" t="n">
-        <v>0.06153371714128571</v>
+        <v>0.06156904481687362</v>
       </c>
       <c r="G18" t="n">
-        <v>16.15094145124501</v>
+        <v>16.11685158682197</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1079,13 +1079,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2.168929766152869</v>
+        <v>2.247937012148917</v>
       </c>
       <c r="F20" t="n">
-        <v>0.2044488767180298</v>
+        <v>0.210768117948621</v>
       </c>
       <c r="G20" t="n">
-        <v>10.60866560364422</v>
+        <v>10.66545089464732</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1149,16 +1149,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1.260391956826582</v>
+        <v>29.06938463022569</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1808345944640299</v>
+        <v>4.12258144150827</v>
       </c>
       <c r="G22" t="n">
-        <v>6.969860830861758</v>
+        <v>7.051257820532816</v>
       </c>
       <c r="H22" t="n">
-        <v>3.172573315168847e-12</v>
+        <v>1.773026170326375e-12</v>
       </c>
     </row>
     <row r="23">
@@ -1219,13 +1219,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.8628411151197651</v>
+        <v>0.8595749847123999</v>
       </c>
       <c r="F24" t="n">
-        <v>0.04857167716009689</v>
+        <v>0.04835879854610016</v>
       </c>
       <c r="G24" t="n">
-        <v>17.76428498151287</v>
+        <v>17.77494500561665</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1251,13 +1251,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1.189796743535845</v>
+        <v>1.190290728935986</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0533145274233466</v>
+        <v>0.05315076725045578</v>
       </c>
       <c r="G25" t="n">
-        <v>22.31655800052187</v>
+        <v>22.3946104729727</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,13 +1283,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1.163769184986943</v>
+        <v>1.165314703426953</v>
       </c>
       <c r="F26" t="n">
-        <v>0.052004636732066</v>
+        <v>0.05187881870989761</v>
       </c>
       <c r="G26" t="n">
-        <v>22.37818121796409</v>
+        <v>22.46224436837781</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1315,13 +1315,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1.049420844987561</v>
+        <v>1.05047581507337</v>
       </c>
       <c r="F27" t="n">
-        <v>0.05017351244934948</v>
+        <v>0.05003889817261487</v>
       </c>
       <c r="G27" t="n">
-        <v>20.91583374845528</v>
+        <v>20.99318437085967</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1347,13 +1347,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.8679728233233112</v>
+        <v>0.8655153626619519</v>
       </c>
       <c r="F28" t="n">
-        <v>0.05018966593001532</v>
+        <v>0.04998533725197549</v>
       </c>
       <c r="G28" t="n">
-        <v>17.29385536290124</v>
+        <v>17.31538507545891</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1379,13 +1379,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1.014172415155218</v>
+        <v>1.014766433664062</v>
       </c>
       <c r="F29" t="n">
-        <v>0.05175320670365571</v>
+        <v>0.05160365669807751</v>
       </c>
       <c r="G29" t="n">
-        <v>19.59632030036089</v>
+        <v>19.664622597999</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1449,13 +1449,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1.056941536439403</v>
+        <v>1.056851642486047</v>
       </c>
       <c r="F31" t="n">
-        <v>0.06242996139864623</v>
+        <v>0.06239364270168985</v>
       </c>
       <c r="G31" t="n">
-        <v>16.93003668019875</v>
+        <v>16.93845072521282</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1481,13 +1481,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1.36649057091997</v>
+        <v>1.365019161272189</v>
       </c>
       <c r="F32" t="n">
-        <v>0.06608187033260619</v>
+        <v>0.06596052473654311</v>
       </c>
       <c r="G32" t="n">
-        <v>20.67875143396231</v>
+        <v>20.69448608396612</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1513,13 +1513,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1.471575514928222</v>
+        <v>1.470231000730232</v>
       </c>
       <c r="F33" t="n">
-        <v>0.07210849863644854</v>
+        <v>0.07197749824432419</v>
       </c>
       <c r="G33" t="n">
-        <v>20.40779579016196</v>
+        <v>20.42625871378826</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1.090366882267388</v>
+        <v>1.089930520351829</v>
       </c>
       <c r="F34" t="n">
-        <v>0.05796520644723983</v>
+        <v>0.05787890344440328</v>
       </c>
       <c r="G34" t="n">
-        <v>18.81071334130474</v>
+        <v>18.83122269895718</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1577,13 +1577,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1.070264105150613</v>
+        <v>1.070165427913044</v>
       </c>
       <c r="F35" t="n">
-        <v>0.059439167015791</v>
+        <v>0.05937126771221938</v>
       </c>
       <c r="G35" t="n">
-        <v>18.00604145156129</v>
+        <v>18.02497182782515</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1609,13 +1609,13 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1.014433466763671</v>
+        <v>1.014056748276091</v>
       </c>
       <c r="F36" t="n">
-        <v>0.05624832176791955</v>
+        <v>0.05618612272863861</v>
       </c>
       <c r="G36" t="n">
-        <v>18.03491081798292</v>
+        <v>18.04817095416282</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1641,13 +1641,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1.179979581237576</v>
+        <v>1.17797638028677</v>
       </c>
       <c r="F37" t="n">
-        <v>0.06641649487372717</v>
+        <v>0.06631219011744829</v>
       </c>
       <c r="G37" t="n">
-        <v>17.76636336294499</v>
+        <v>17.76410005735963</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -1673,13 +1673,13 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>-0.1243471080785969</v>
+        <v>-0.1245982625728233</v>
       </c>
       <c r="F38" t="n">
-        <v>0.01178301211022364</v>
+        <v>0.01179406600795666</v>
       </c>
       <c r="G38" t="n">
-        <v>-10.55308327826914</v>
+        <v>-10.56448747007188</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -1705,13 +1705,13 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.282903469709996</v>
+        <v>0.2832397078459041</v>
       </c>
       <c r="F39" t="n">
-        <v>0.02543436702050076</v>
+        <v>0.0254361729937514</v>
       </c>
       <c r="G39" t="n">
-        <v>11.12288225890763</v>
+        <v>11.13531142850573</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1737,16 +1737,16 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.08497142177446459</v>
+        <v>0.0840280873982925</v>
       </c>
       <c r="F40" t="n">
-        <v>0.02024640541874096</v>
+        <v>0.02026591795219459</v>
       </c>
       <c r="G40" t="n">
-        <v>4.1968645798041</v>
+        <v>4.146275909749592</v>
       </c>
       <c r="H40" t="n">
-        <v>2.70635644450401e-05</v>
+        <v>3.379265888758809e-05</v>
       </c>
     </row>
     <row r="41">
@@ -1769,13 +1769,13 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.5645205121789726</v>
+        <v>0.5668150737126377</v>
       </c>
       <c r="F41" t="n">
-        <v>0.04547489947434107</v>
+        <v>0.04554407907380634</v>
       </c>
       <c r="G41" t="n">
-        <v>12.41389247017656</v>
+        <v>12.44541738963789</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1801,16 +1801,16 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>-0.03156892494213621</v>
+        <v>-0.02587932929892739</v>
       </c>
       <c r="F42" t="n">
-        <v>0.004567243411075925</v>
+        <v>0.004236697318068256</v>
       </c>
       <c r="G42" t="n">
-        <v>-6.912030319791374</v>
+        <v>-6.108373421544974</v>
       </c>
       <c r="H42" t="n">
-        <v>4.777733764171899e-12</v>
+        <v>1.006516425761106e-09</v>
       </c>
     </row>
     <row r="43">
@@ -1833,16 +1833,16 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.0193101142815962</v>
+        <v>0.01865602317860907</v>
       </c>
       <c r="F43" t="n">
-        <v>0.005523572542171442</v>
+        <v>0.005331593126930251</v>
       </c>
       <c r="G43" t="n">
-        <v>3.495946532913462</v>
+        <v>3.499146077159759</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0004723833432631608</v>
+        <v>0.0004667507946938265</v>
       </c>
     </row>
     <row r="44">
@@ -1865,13 +1865,13 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.5488866625078934</v>
+        <v>0.5487933450345628</v>
       </c>
       <c r="F44" t="n">
-        <v>0.05117507831326135</v>
+        <v>0.05118080997970651</v>
       </c>
       <c r="G44" t="n">
-        <v>10.72566336170962</v>
+        <v>10.7226389195763</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -1897,16 +1897,16 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.1083816632254438</v>
+        <v>0.07459076712668751</v>
       </c>
       <c r="F45" t="n">
-        <v>0.01789004484311935</v>
+        <v>0.01255429587966202</v>
       </c>
       <c r="G45" t="n">
-        <v>6.05821081891083</v>
+        <v>5.941453653452855</v>
       </c>
       <c r="H45" t="n">
-        <v>1.376439184852529e-09</v>
+        <v>2.825056188981989e-09</v>
       </c>
     </row>
     <row r="46">
@@ -1929,13 +1929,13 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.2712627419736816</v>
+        <v>0.2716663899165763</v>
       </c>
       <c r="F46" t="n">
-        <v>0.02177776252147423</v>
+        <v>0.02179934986194294</v>
       </c>
       <c r="G46" t="n">
-        <v>12.45595095886199</v>
+        <v>12.46213266104721</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -1961,13 +1961,13 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.4111899455033919</v>
+        <v>0.4115037958363476</v>
       </c>
       <c r="F47" t="n">
-        <v>0.01772709083181419</v>
+        <v>0.0177375935546514</v>
       </c>
       <c r="G47" t="n">
-        <v>23.19556826223556</v>
+        <v>23.19952785845845</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -1993,13 +1993,13 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.2278487412997965</v>
+        <v>0.2286175082404036</v>
       </c>
       <c r="F48" t="n">
-        <v>0.01125186647420467</v>
+        <v>0.01127447684755106</v>
       </c>
       <c r="G48" t="n">
-        <v>20.24986181642827</v>
+        <v>20.27743826267064</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -2025,13 +2025,13 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.3889868244383897</v>
+        <v>0.3891523076401167</v>
       </c>
       <c r="F49" t="n">
-        <v>0.01725747377224602</v>
+        <v>0.01725698927942816</v>
       </c>
       <c r="G49" t="n">
-        <v>22.54019502213758</v>
+        <v>22.55041718554405</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -2057,13 +2057,13 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.5744482286578751</v>
+        <v>0.5739326868901039</v>
       </c>
       <c r="F50" t="n">
-        <v>0.02493333585758538</v>
+        <v>0.02490604376301568</v>
       </c>
       <c r="G50" t="n">
-        <v>23.03936512610981</v>
+        <v>23.0439122458832</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.7776426324739637</v>
+        <v>0.7789431947838795</v>
       </c>
       <c r="F51" t="n">
-        <v>0.03317836920807585</v>
+        <v>0.03321877257666887</v>
       </c>
       <c r="G51" t="n">
-        <v>23.43824157159725</v>
+        <v>23.44888550480398</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -2121,16 +2121,16 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.1442050328153552</v>
+        <v>0.1808331222339894</v>
       </c>
       <c r="F52" t="n">
-        <v>0.01747711024091637</v>
+        <v>0.01316062605541751</v>
       </c>
       <c r="G52" t="n">
-        <v>8.251079887881</v>
+        <v>13.74046504009661</v>
       </c>
       <c r="H52" t="n">
-        <v>2.220446049250313e-16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2153,13 +2153,13 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.5111090843701376</v>
+        <v>0.5106929001005475</v>
       </c>
       <c r="F53" t="n">
-        <v>0.02191123267828708</v>
+        <v>0.02188856265959852</v>
       </c>
       <c r="G53" t="n">
-        <v>23.32635008952711</v>
+        <v>23.33149544898364</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -2185,13 +2185,13 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.4867919021906887</v>
+        <v>0.4867814007794727</v>
       </c>
       <c r="F54" t="n">
-        <v>0.02400383226479211</v>
+        <v>0.02398743357143409</v>
       </c>
       <c r="G54" t="n">
-        <v>20.27975769870782</v>
+        <v>20.29318390020985</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -2217,13 +2217,13 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.6171928963086853</v>
+        <v>0.6166916282316307</v>
       </c>
       <c r="F55" t="n">
-        <v>0.02980199811839837</v>
+        <v>0.02976632818113006</v>
       </c>
       <c r="G55" t="n">
-        <v>20.709782405729</v>
+        <v>20.71775949180913</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.5313849016302371</v>
+        <v>0.5308005535915546</v>
       </c>
       <c r="F56" t="n">
-        <v>0.0237368829445691</v>
+        <v>0.02370572271501438</v>
       </c>
       <c r="G56" t="n">
-        <v>22.38646509942997</v>
+        <v>22.39124113406476</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -2281,13 +2281,13 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.6234203468854654</v>
+        <v>0.6231962515807737</v>
       </c>
       <c r="F57" t="n">
-        <v>0.02720869384152489</v>
+        <v>0.02719179739571496</v>
       </c>
       <c r="G57" t="n">
-        <v>22.91254223718421</v>
+        <v>22.91853835510197</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -2313,13 +2313,13 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.5562564067956561</v>
+        <v>0.5564980187624257</v>
       </c>
       <c r="F58" t="n">
-        <v>0.02429494417743227</v>
+        <v>0.02429567224759274</v>
       </c>
       <c r="G58" t="n">
-        <v>22.89597385819352</v>
+        <v>22.90523238329655</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -2345,13 +2345,13 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.8016375396848844</v>
+        <v>0.8026604481772592</v>
       </c>
       <c r="F59" t="n">
-        <v>0.03478649327708712</v>
+        <v>0.03480482215443185</v>
       </c>
       <c r="G59" t="n">
-        <v>23.04450561534054</v>
+        <v>23.06175979273008</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -2377,13 +2377,13 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.2744256616865078</v>
+        <v>0.2743364102508545</v>
       </c>
       <c r="F60" t="n">
-        <v>0.01314998362180026</v>
+        <v>0.01314532221921453</v>
       </c>
       <c r="G60" t="n">
-        <v>20.86889760156748</v>
+        <v>20.86950822924577</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -2409,13 +2409,13 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.1660462167855502</v>
+        <v>0.16575240983025</v>
       </c>
       <c r="F61" t="n">
-        <v>0.009649167261881248</v>
+        <v>0.009643725215519643</v>
       </c>
       <c r="G61" t="n">
-        <v>17.20834682017614</v>
+        <v>17.18759152804532</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -2441,13 +2441,13 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.7412356275220363</v>
+        <v>0.7406292544172742</v>
       </c>
       <c r="F62" t="n">
-        <v>0.03349051030140342</v>
+        <v>0.03345090671820029</v>
       </c>
       <c r="G62" t="n">
-        <v>22.13270627497253</v>
+        <v>22.14078262913468</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -2473,13 +2473,13 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.8675518054467378</v>
+        <v>0.8679840841599217</v>
       </c>
       <c r="F63" t="n">
-        <v>0.03723745909622696</v>
+        <v>0.03721328401337765</v>
       </c>
       <c r="G63" t="n">
-        <v>23.29782499878849</v>
+        <v>23.32457634818172</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -2505,13 +2505,13 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.6081500412406353</v>
+        <v>0.6073580199410202</v>
       </c>
       <c r="F64" t="n">
-        <v>0.03072347825016555</v>
+        <v>0.0306847284708308</v>
       </c>
       <c r="G64" t="n">
-        <v>19.79430962435264</v>
+        <v>19.79349501165009</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2537,13 +2537,13 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.571867838205361</v>
+        <v>0.5712264637194502</v>
       </c>
       <c r="F65" t="n">
-        <v>0.02903174875905907</v>
+        <v>0.02901429736155219</v>
       </c>
       <c r="G65" t="n">
-        <v>19.69801553918509</v>
+        <v>19.68775795538353</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -2569,13 +2569,13 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.6714998584567935</v>
+        <v>0.6709012550281609</v>
       </c>
       <c r="F66" t="n">
-        <v>0.03132291508153651</v>
+        <v>0.03129580016735866</v>
       </c>
       <c r="G66" t="n">
-        <v>21.43797461658271</v>
+        <v>21.43742136066135</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2601,13 +2601,13 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.9601718833074322</v>
+        <v>0.960147549742732</v>
       </c>
       <c r="F67" t="n">
-        <v>0.04090815724496384</v>
+        <v>0.04087088830626228</v>
       </c>
       <c r="G67" t="n">
-        <v>23.47140394357818</v>
+        <v>23.49221143725729</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2633,13 +2633,13 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.8343238489095083</v>
+        <v>0.8338111032419483</v>
       </c>
       <c r="F68" t="n">
-        <v>0.03723056556254582</v>
+        <v>0.03719870917906354</v>
       </c>
       <c r="G68" t="n">
-        <v>22.40964745715369</v>
+        <v>22.41505475918033</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -2665,13 +2665,13 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.7326536250451668</v>
+        <v>0.7311740188316894</v>
       </c>
       <c r="F69" t="n">
-        <v>0.04160359630836381</v>
+        <v>0.04161329502409861</v>
       </c>
       <c r="G69" t="n">
-        <v>17.61034357696301</v>
+        <v>17.57068308074835</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -2697,13 +2697,13 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.6833517708044319</v>
+        <v>0.6870958936074285</v>
       </c>
       <c r="F70" t="n">
-        <v>0.05705372178684578</v>
+        <v>0.05713111553432233</v>
       </c>
       <c r="G70" t="n">
-        <v>11.97733906554729</v>
+        <v>12.02664935157129</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -2729,13 +2729,13 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.8659541212946323</v>
+        <v>0.867195640879427</v>
       </c>
       <c r="F71" t="n">
-        <v>0.04541273318124307</v>
+        <v>0.0454397542371307</v>
       </c>
       <c r="G71" t="n">
-        <v>19.06853123813369</v>
+        <v>19.08451432934294</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -2761,13 +2761,13 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.5188188738076706</v>
+        <v>88.70895208523277</v>
       </c>
       <c r="F72" t="n">
-        <v>0.0333039950046146</v>
+        <v>9.976332187242079</v>
       </c>
       <c r="G72" t="n">
-        <v>15.57827743248835</v>
+        <v>8.891940486771936</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
@@ -2793,13 +2793,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.1339699788588705</v>
+        <v>0.1354811666211702</v>
       </c>
       <c r="F73" t="n">
-        <v>0.007464627955808155</v>
+        <v>0.007372212836189067</v>
       </c>
       <c r="G73" t="n">
-        <v>17.94730824282843</v>
+        <v>18.3772728233966</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.9466619878038232</v>
+        <v>0.9380783547669456</v>
       </c>
       <c r="F74" t="n">
-        <v>0.04485697123621937</v>
+        <v>0.04504950383643331</v>
       </c>
       <c r="G74" t="n">
-        <v>21.10401040671121</v>
+        <v>20.82327827964803</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>

</xml_diff>